<commit_message>
fix: adjust app api
</commit_message>
<xml_diff>
--- a/excel/appkpi.xlsx
+++ b/excel/appkpi.xlsx
@@ -175,11 +175,13 @@
   </si>
   <si>
     <t xml:space="preserve">描述：
-统计当月产生或激活，且未解决的bug，每个扣0.4分</t>
+统计当月产生或激活，且未解决的bug
+严重bug(严重程度1级与2级)，1个扣0.6分
+一般bug(3级以上)，扣0.4分</t>
   </si>
   <si>
     <t xml:space="preserve">
-分值=25 – (当月bug数)*0.4</t>
+分值=25 – (当月严重bug数)*0.6 – (当月一般bug数)*0.4</t>
   </si>
   <si>
     <t xml:space="preserve">团队协作
@@ -887,7 +889,7 @@
         <v>16</v>
       </c>
       <c r="D5" s="10" t="n">
-        <v>0.35</v>
+        <v>0.3</v>
       </c>
       <c r="E5" s="11" t="s">
         <v>17</v>
@@ -905,7 +907,7 @@
         <v>19</v>
       </c>
       <c r="D6" s="10" t="n">
-        <v>0.25</v>
+        <v>0.3</v>
       </c>
       <c r="E6" s="11" t="s">
         <v>20</v>

</xml_diff>

<commit_message>
fix: adjust app kpi template
</commit_message>
<xml_diff>
--- a/excel/appkpi.xlsx
+++ b/excel/appkpi.xlsx
@@ -170,8 +170,7 @@
     <t xml:space="preserve">分值=当月完成需求分值总和（需求状态是研发完毕）</t>
   </si>
   <si>
-    <t xml:space="preserve">项目平均
-bug关闭率</t>
+    <t xml:space="preserve">bug遗留数</t>
   </si>
   <si>
     <t xml:space="preserve">描述：
@@ -181,7 +180,7 @@
   </si>
   <si>
     <t xml:space="preserve">
-分值=25 – (当月严重bug数)*0.6 – (当月一般bug数)*0.4</t>
+分值=30 – (当月严重bug数)*0.6 – (当月一般bug数)*0.4</t>
   </si>
   <si>
     <t xml:space="preserve">团队协作

</xml_diff>